<commit_message>
Update tracker and structure doc with confirmed owners and details
- Name Feron (commercial) and Jason (product) as leads / sign-off.
- Two gaps: owner marked TBD (not Kelly); add explicit Session 3
  agenda item to assign an owner.
- SharePoint roadmap: Kelly has access; Jason to commit Product team
  to maintain it.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012kg3Y6dfNgYmGi2er96sJG
</commit_message>
<xml_diff>
--- a/Product_Commercial_Tracker.xlsx
+++ b/Product_Commercial_Tracker.xlsx
@@ -638,12 +638,12 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Confirm folder location &amp; that Product will keep it updated</t>
+          <t>Jason to commit Product team to keep it updated</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -653,7 +653,7 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Kelly coordinates access; Product owns content</t>
+          <t>Kelly has folder access; Jason committing Product team to maintain content</t>
         </is>
       </c>
     </row>
@@ -925,7 +925,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Agree owner at next meeting</t>
+          <t>Assign an owner at Session 3</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Identified gap — no owner yet</t>
+          <t>Identified gap — no owner yet. TBD (not Kelly)</t>
         </is>
       </c>
     </row>
@@ -972,7 +972,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Agree owner &amp; format (visual + commentary)</t>
+          <t>Assign an owner at Session 3; agree format</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -982,7 +982,7 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Identified gap; possible AI-assisted approach</t>
+          <t>Identified gap; possible AI-assisted approach. TBD (not Kelly)</t>
         </is>
       </c>
     </row>
@@ -1113,7 +1113,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Share this workbook + structure doc</t>
+          <t>Share workbook + structure doc; sign-off from Feron &amp; Jason</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Kelly's deliverable</t>
+          <t>Kelly's deliverable; leads = Feron (commercial) &amp; Jason (product)</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Two identified gaps with no owner</t>
+          <t>Two identified gaps with no owner (not Kelly)</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Agree owners at Session 3</t>
+          <t>Session 3 agenda item: assign an owner</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Apply Kiron green/black palette to tables
Replace blue with Kiron branding: dark green headers, black title bar,
bright green accents and light green row shading, in both the OneNote
HTML tables and the tracker spreadsheet.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012kg3Y6dfNgYmGi2er96sJG
</commit_message>
<xml_diff>
--- a/Product_Commercial_Tracker.xlsx
+++ b/Product_Commercial_Tracker.xlsx
@@ -66,12 +66,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="00111111"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E5496"/>
+        <fgColor rgb="000B5D2E"/>
       </patternFill>
     </fill>
     <fill>

</xml_diff>

<commit_message>
Remove ID columns; link commercial requests by roadmap item name
Drop the ID column from all tables in both the OneNote HTML and the
tracker spreadsheet. Replace the Commercial Requests 'Linked ID' column
with 'Linked Roadmap Item', naming the product/feature so the connection
still holds without IDs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012kg3Y6dfNgYmGi2er96sJG
</commit_message>
<xml_diff>
--- a/Product_Commercial_Tracker.xlsx
+++ b/Product_Commercial_Tracker.xlsx
@@ -488,18 +488,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -519,45 +518,40 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>Action / Topic</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Action / Topic</t>
+          <t>Raised in Meeting</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Raised in Meeting</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Priority</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Priority</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Next Step</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Next Step</t>
+          <t>Target / Due</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Target / Due</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -566,45 +560,40 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>EX</t>
+          <t>EXAMPLE — Confirm Q3 Plinko release date with Product</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>EXAMPLE — Confirm Q3 Plinko release date with Product</t>
+          <t>Sep 2026 (Session 2)</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Sep 2026 (Session 2)</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Product to confirm target quarter</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Product to confirm target quarter</t>
+          <t>Next meeting</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>Next meeting</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Example row — delete before use</t>
         </is>
@@ -613,92 +602,82 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>Product roadmap accessible via Global Product SharePoint folder (status + target dates)</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Product roadmap accessible via Global Product SharePoint folder (status + target dates)</t>
+          <t>Session 2</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Session 2</t>
+          <t>Facilitator</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Kelly</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Jason to commit Product team to keep it updated</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Jason to commit Product team to keep it updated</t>
+          <t>Before Sess. 3</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Before Sess. 3</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>Kelly has folder access; Jason committing Product team to maintain content</t>
+          <t>Facilitator has folder access; Jason committing Product team to maintain content</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>Establish action/roadmap follow-up so each meeting reviews prior items</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Establish action/roadmap follow-up so each meeting reviews prior items</t>
+          <t>Session 2</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Session 2</t>
+          <t>Facilitator</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Kelly</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Stand up this tracker + share with group</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Stand up this tracker + share with group</t>
+          <t>Before Sess. 3</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>Before Sess. 3</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>This workbook</t>
         </is>
@@ -707,92 +686,82 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>Share product demos/visuals so Commercial can prepare (e.g. cricket roulette demo from Josh)</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Share product demos/visuals so Commercial can prepare (e.g. cricket roulette demo from Josh)</t>
+          <t>Session 2</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Session 2</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Product to circulate available demos</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Product to circulate available demos</t>
+          <t>Ongoing</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>Josh has cricket roulette demo; Kelly to request</t>
+          <t>Josh has cricket roulette demo</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>Astro → Betman integration plan</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Astro → Betman integration plan</t>
+          <t>Session 2</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Session 2</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Confirm approach &amp; rough timing</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Product to confirm approach &amp; rough timing</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>Jason flagged as a specific requirement</t>
         </is>
@@ -801,45 +770,40 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>Third-party games — strategic review + business case (continue or not, outside Aviator)</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Third-party games — strategic review + business case (continue or not, outside Aviator)</t>
+          <t>Session 2</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Session 2</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Commercial</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Review Paul's earlier analysis; commercial to build case</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Review Paul's earlier analysis; commercial to build case</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>Needs decision + possible dedicated resource</t>
         </is>
@@ -848,45 +812,40 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>Mobile POS / retail opportunity — commercial validation before final decision</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Mobile POS / retail opportunity — commercial validation before final decision</t>
+          <t>Session 2</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Session 2</t>
+          <t>Retail team</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Retail team</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Retail (Dieg/Tony/Tom) to finalise business case w/ data</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Retail (Dieg/Tony/Tom) to finalise business case w/ data</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>East Africa / Golden Race competitive pressure</t>
         </is>
@@ -895,139 +854,124 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>A7</t>
+          <t>Competitive product analysis (our products vs competitors) — agree owner &amp; scope</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Competitive product analysis (our products vs competitors) — agree owner &amp; scope</t>
+          <t>Session 2</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Session 2</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Assign an owner at Session 3</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Assign an owner at Session 3</t>
+          <t>Sess. 3</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Sess. 3</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>Identified gap — no owner yet. TBD (not Kelly)</t>
+          <t>Identified gap — no owner yet. TBD (not Facilitator)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>A8</t>
+          <t>Insight-driven product performance view (narrative, not just Power BI)</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Insight-driven product performance view (narrative, not just Power BI)</t>
+          <t>Session 2</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Session 2</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Assign an owner at Session 3; agree format</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Assign an owner at Session 3; agree format</t>
+          <t>Sess. 3</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Sess. 3</t>
-        </is>
-      </c>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>Identified gap; possible AI-assisted approach. TBD (not Kelly)</t>
+          <t>Identified gap; possible AI-assisted approach. TBD (not Facilitator)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>A9</t>
+          <t>Link GTM / customer comms more closely to upcoming releases</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Link GTM / customer comms more closely to upcoming releases</t>
+          <t>Session 2</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Session 2</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Commercial</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Feed into Patrick's GTM board</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Feed into Patrick's GTM board</t>
+          <t>Ongoing</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>Philip/Josh/Jade → Patrick's board</t>
         </is>
@@ -1036,45 +980,40 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>A10</t>
+          <t>Share recent football / cinematic updates with team + marketing</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Share recent football / cinematic updates with team + marketing</t>
+          <t>Session 2</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Session 2</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Product to send footage; confirm in marketing assets</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Product to send footage; confirm in marketing assets</t>
+          <t>Before Sess. 3</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>Before Sess. 3</t>
-        </is>
-      </c>
-      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>Sarah requested; Jason has video</t>
         </is>
@@ -1083,92 +1022,82 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>A11</t>
+          <t>Propose meeting structure / action-tracking to group for input</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Propose meeting structure / action-tracking to group for input</t>
+          <t>Session 2</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Session 2</t>
+          <t>Facilitator</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Kelly</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Share workbook + structure doc; sign-off from Feron &amp; Jason</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Share workbook + structure doc; sign-off from Feron &amp; Jason</t>
+          <t>Before Sess. 3</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Before Sess. 3</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>Kelly's deliverable; leads = Feron (commercial) &amp; Jason (product)</t>
+          <t>Leads = Feron (commercial) &amp; Jason (product)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>A12</t>
+          <t>Schedule next monthly session (proposed 18 Sep, 11:00–12:00)</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Schedule next monthly session (proposed 18 Sep, 11:00–12:00)</t>
+          <t>Session 2</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Session 2</t>
+          <t>Facilitator</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Kelly</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Confirm availability, send invite</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Confirm availability, send invite</t>
+          <t>18 Sep</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>18 Sep</t>
-        </is>
-      </c>
-      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Awaiting confirmations</t>
         </is>
@@ -1176,17 +1105,17 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <dataValidations count="3">
+    <dataValidation sqref="C4:C57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Facilitator,Product,Commercial,Marketing,Retail team,TBD"</formula1>
+    </dataValidation>
     <dataValidation sqref="D4:D57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Kelly,Product,Commercial,Marketing,Retail team,TBD"</formula1>
+      <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
     <dataValidation sqref="E4:E57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"High,Medium,Low"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F4:F57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In Progress,Blocked,Done,Parked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1200,18 +1129,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1231,45 +1159,40 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>Channel</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Channel</t>
+          <t>Product / Feature</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Product / Feature</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Stage</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Stage</t>
+          <t>Target Release</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Target Release</t>
+          <t>Commercial Angle</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Commercial Angle</t>
+          <t>Status Change</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Status Change</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Updated</t>
         </is>
@@ -1278,45 +1201,40 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>EX</t>
+          <t>VSE</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>VSE</t>
+          <t>EXAMPLE — New race track pack</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>EXAMPLE — New race track pack</t>
+          <t>Additional dirt/turf tracks for Betmakers global launch</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Additional dirt/turf tracks for Betmakers global launch</t>
+          <t>Concept</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Q4 2026</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Q4 2026</t>
+          <t>Variety for global distribution</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Variety for global distribution</t>
+          <t>New</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Example</t>
         </is>
@@ -1325,45 +1243,40 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>VSE</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>VSE</t>
+          <t>One-minute horse racing (sprint)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>One-minute horse racing (sprint)</t>
+          <t>Shorter event envelope following Entain success; English-look sprint product</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Shorter event envelope following Entain success; English-look sprint product</t>
+          <t>In Dev</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>In Dev</t>
+          <t>ASAP</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>ASAP</t>
+          <t>Match Entain need; roll across all online racing</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Match Entain need; roll across all online racing</t>
+          <t>Priority</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>Sep 2026</t>
         </is>
@@ -1372,45 +1285,40 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>VSE</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>VSE</t>
+          <t>Sprint dog racing</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Sprint dog racing</t>
+          <t>Switch dog racing to shorter single-loop format</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Switch dog racing to shorter single-loop format</t>
+          <t>Concept</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Consistency with sprint racing</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Consistency with sprint racing</t>
+          <t>New</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>Sep 2026</t>
         </is>
@@ -1419,45 +1327,40 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>VSE</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>VSE</t>
+          <t>Faster football (1-min envelope)</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Faster football (1-min envelope)</t>
+          <t>6-goal game completing within one minute</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>6-goal game completing within one minute</t>
+          <t>In Dev</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>In Dev</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>1-min game intervals online</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>1-min game intervals online</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>Sep 2026</t>
         </is>
@@ -1466,45 +1369,40 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>P4</t>
+          <t>VSE</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>VSE</t>
+          <t>New race tracks (variety)</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>New race tracks (variety)</t>
+          <t>6–8 tracks incl. more dirt for US/global</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>6–8 tracks incl. more dirt for US/global</t>
+          <t>Concept</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Post-Betmakers</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Post-Betmakers</t>
+          <t>Needed for Betmakers global deal</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Needed for Betmakers global deal</t>
+          <t>New</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>Sep 2026</t>
         </is>
@@ -1513,45 +1411,40 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>VSE</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>VSE</t>
+          <t>Racing visuals refresh</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Racing visuals refresh</t>
+          <t>Modernised preamble/results, more energetic horse animation</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Modernised preamble/results, more energetic horse animation</t>
+          <t>In Dev</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>In Dev</t>
+          <t>With sprint</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>With sprint</t>
+          <t>Refresh vs 2015-era look</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Refresh vs 2015-era look</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>Sep 2026</t>
         </is>
@@ -1560,45 +1453,40 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>P6</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>Italian 3-goal micro-betting football</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Italian 3-goal micro-betting football</t>
+          <t>Header/penalty/L-R foot/save micro events</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Header/penalty/L-R foot/save micro events</t>
+          <t>In Dev</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>In Dev</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Italian operators keen</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Italian operators keen</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>Sep 2026</t>
         </is>
@@ -1607,45 +1495,40 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>P7</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>iGoal / Bet Power</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>iGoal / Bet Power</t>
+          <t>Sustained-revenue instant football; strong margin</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Sustained-revenue instant football; strong margin</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Live</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>Retains revenue vs slots</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Retains revenue vs slots</t>
+          <t>Stable</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>Stable</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
         <is>
           <t>Sep 2026</t>
         </is>
@@ -1654,45 +1537,40 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>P8</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>'Hop' — new math game</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>'Hop' — new math game</t>
+          <t>Original simple math-based instant game</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Original simple math-based instant game</t>
+          <t>Concept</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>After racing</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>After racing</t>
+          <t>New original IP</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>New original IP</t>
+          <t>New</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>Sep 2026</t>
         </is>
@@ -1701,45 +1579,40 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>P9</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>Cricket roulette</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Cricket roulette</t>
+          <t>Demo available (Josh) — target Stake</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Demo available (Josh) — target Stake</t>
+          <t>Concept</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Steven pushing to Stake</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Steven pushing to Stake</t>
+          <t>Demo ready</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>Demo ready</t>
-        </is>
-      </c>
-      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>Sep 2026</t>
         </is>
@@ -1748,45 +1621,40 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>Betman</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Betman</t>
+          <t>Mobile / retail wallet</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Mobile / retail wallet</t>
+          <t>Voucher-based play across terminals &amp; mobile in-venue</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Voucher-based play across terminals &amp; mobile in-venue</t>
+          <t>Staging</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Staging</t>
+          <t>Post v6</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Post v6</t>
+          <t>Transformative for African retail</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Transformative for African retail</t>
+          <t>New release</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>New release</t>
-        </is>
-      </c>
-      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>Sep 2026</t>
         </is>
@@ -1795,45 +1663,40 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>Betman</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Betman</t>
+          <t>Vision X + Net4Media (racing)</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Vision X + Net4Media (racing)</t>
+          <t>Horse then dog racing on Net4Media to cut bandwidth</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Horse then dog racing on Net4Media to cut bandwidth</t>
+          <t>Concept</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Bandwidth-light shop content</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Bandwidth-light shop content</t>
+          <t>Next up</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>Next up</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>Sep 2026</t>
         </is>
@@ -1842,45 +1705,40 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>P12</t>
+          <t>Betman</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Betman</t>
+          <t>Football cinematic close-ups</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Football cinematic close-ups</t>
+          <t>New close-up/replay sequences; multilingual soccer</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>New close-up/replay sequences; multilingual soccer</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Live</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>Marketing asset for customers</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Marketing asset for customers</t>
+          <t>Recently shipped</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>Recently shipped</t>
-        </is>
-      </c>
-      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Sep 2026</t>
         </is>
@@ -1888,14 +1746,14 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="B4:B47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A4:A57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"VSE,Instant,Betman,Cross"</formula1>
     </dataValidation>
-    <dataValidation sqref="E4:E47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D4:D57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Concept,In Dev,Staging,Production,Parked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1909,19 +1767,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1934,57 +1791,52 @@
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>HOW TO USE:  Commercial logs what customers/markets are asking for. Link to a Product Roadmap ID where relevant. This is the 'two-way' input the meeting is built around.</t>
+          <t>HOW TO USE:  Commercial logs what customers/markets are asking for. Name the linked roadmap item so the connection holds. This is the 'two-way' input the meeting is built around.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>Date Raised</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Date Raised</t>
+          <t>Customer / Market</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Customer / Market</t>
+          <t>Tier</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Tier</t>
+          <t>Request / Feedback</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Request / Feedback</t>
+          <t>Product Area</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Product Area</t>
+          <t>Linked Roadmap Item</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Linked Roadmap ID</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1993,50 +1845,45 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>EX</t>
+          <t>01 Sep 26</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>01 Sep 26</t>
+          <t>Betway (SA)</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Betway (SA)</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>EXAMPLE — Interested in Plinko-style game</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>EXAMPLE — Interested in Plinko-style game</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>→ (name the roadmap item)</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>Commercial</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Example row — delete before use</t>
         </is>
@@ -2045,50 +1892,45 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>Sep 26</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Sep 26</t>
+          <t>Third-party game clients</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Third-party game clients</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Want newest Astro / ESA / other third-party games distributed</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Want newest Astro / ESA / other third-party games distributed</t>
+          <t>Betman</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Betman</t>
+          <t>→ Astro → Betman integration</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>P-Astro</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>Commercial</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>Blocked on Betman integration</t>
         </is>
@@ -2097,102 +1939,92 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>Sep 26</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Sep 26</t>
+          <t>Ethiopia market</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Ethiopia market</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
+          <t>Market entry — third-party (Galaxis/Smartsoft/Split the Pot) interest</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Cross</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Market entry — third-party (Galaxis/Smartsoft/Split the Pot) interest</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Cross</t>
-        </is>
-      </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Parked</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Parked</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Commercial</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>Prove payment first (Jason) before more games</t>
+          <t>Prove payment first before more games</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>Sep 26</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Sep 26</t>
+          <t>Italian operators</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Italian operators</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Keen on 3-goal micro-betting football</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Keen on 3-goal micro-betting football</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>→ Italian 3-goal micro-betting football</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>P6</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>Commercial</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>Salivating per Jason</t>
         </is>
@@ -2201,50 +2033,45 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>Sep 26</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Sep 26</t>
+          <t>East Africa retail</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>East Africa retail</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Retail solution to counter Golden Race</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Retail solution to counter Golden Race</t>
+          <t>Betman</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Betman</t>
+          <t>→ Mobile POS / retail opportunity</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Retail team</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>Retail team</t>
-        </is>
-      </c>
-      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>Mobile POS business case</t>
         </is>
@@ -2252,21 +2079,21 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation sqref="D4:D49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C4:C49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Tier 1,Tier 2,Tier 3,—"</formula1>
     </dataValidation>
-    <dataValidation sqref="F4:F49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4:E49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"VSE,Instant,Betman,Cross"</formula1>
     </dataValidation>
-    <dataValidation sqref="H4:H49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G4:G49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In Progress,Blocked,Done,Parked"</formula1>
     </dataValidation>
-    <dataValidation sqref="I4:I49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Kelly,Product,Commercial,Marketing,Retail team,TBD"</formula1>
+    <dataValidation sqref="H4:H49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Facilitator,Product,Commercial,Marketing,Retail team,TBD"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2279,17 +2106,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -2309,40 +2135,35 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Detail</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Detail</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Decision / Answer</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Decision / Answer</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
@@ -2351,40 +2172,35 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>EX</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>EXAMPLE — Continue third-party slots?</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>EXAMPLE — Continue third-party slots?</t>
+          <t>Whether to endure beyond proof-of-concept</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Whether to endure beyond proof-of-concept</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Commercial</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Pending business case</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Pending business case</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Example</t>
         </is>
@@ -2393,40 +2209,35 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Question</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Question</t>
+          <t>Do we continue third-party games (outside Aviator)?</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Do we continue third-party games (outside Aviator)?</t>
+          <t>Thin margins; needs dedicated resource + channel</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Thin margins; needs dedicated resource + channel</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Commercial</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Awaiting business case &amp; commercial decision</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>Awaiting business case &amp; commercial decision</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Sep 26</t>
         </is>
@@ -2435,40 +2246,35 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Question</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Question</t>
+          <t>Do we stay in East Africa retail?</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Do we stay in East Africa retail?</t>
+          <t>Golden Race pressure; mobile POS viability</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Golden Race pressure; mobile POS viability</t>
+          <t>Retail team</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Retail team</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Needs data-backed argument</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>Needs data-backed argument</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Sep 26</t>
         </is>
@@ -2477,40 +2283,35 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Question</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Question</t>
+          <t>Who owns competitive analysis + product-performance narrative?</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Who owns competitive analysis + product-performance narrative?</t>
+          <t>Two identified gaps with no owner (not Facilitator)</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Two identified gaps with no owner (not Kelly)</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Session 3 agenda item: assign an owner</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>Session 3 agenda item: assign an owner</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Sep 26</t>
         </is>
@@ -2519,40 +2320,35 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Move to one-minute racing events</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Move to one-minute racing events</t>
+          <t>Testing on Betman OK; move ahead</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Testing on Betman OK; move ahead</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Proceeding — sprint format</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>Proceeding — sprint format</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>Sep 26</t>
         </is>
@@ -2561,40 +2357,35 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Cancel full CG racing revamp</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Cancel full CG racing revamp</t>
+          <t>Poor results vs cost</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Poor results vs cost</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Cancelled; refine current instead</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>Cancelled; refine current instead</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>Sep 26</t>
         </is>
@@ -2603,40 +2394,35 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Decision</t>
+          <t>Ethiopia: prove payment before more games</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Ethiopia: prove payment before more games</t>
+          <t>Sequence risk down</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Sequence risk down</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Commercial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Go live w/ existing, 1 month, then expand</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>Go live w/ existing, 1 month, then expand</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>Sep 26</t>
         </is>
@@ -2644,17 +2430,17 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation sqref="B4:B41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A4:A51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Decision,Question"</formula1>
     </dataValidation>
-    <dataValidation sqref="E4:E41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Kelly,Product,Commercial,Marketing,Retail team,TBD"</formula1>
+    <dataValidation sqref="D4:D51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Facilitator,Product,Commercial,Marketing,Retail team,TBD"</formula1>
     </dataValidation>
-    <dataValidation sqref="F4:F41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4:E51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In Progress,Blocked,Done,Parked"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>